<commit_message>
Add script to list and display .prn files from specified directory
</commit_message>
<xml_diff>
--- a/resultats_crete_a_crete.xlsx
+++ b/resultats_crete_a_crete.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,9 +425,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Nom du fichier</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Valeur crête à crête</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a - Copie.XLSX</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0.08668237445650107</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.08668237445650107</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
No code changes made.
</commit_message>
<xml_diff>
--- a/resultats_crete_a_crete.xlsx
+++ b/resultats_crete_a_crete.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,21 +443,81 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a - Copie.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-a.XLSX</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.08668237445650107</v>
+        <v>0.0229099980453995</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.02831041432609993</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.03152538050700038</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.06183111333809954</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.06250011095490038</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a.XLSX</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B7" t="n">
         <v>0.08668237445650107</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.08219353249770123</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.07733982644349879</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add function to convert .prn files to .xlsx format in convert.py
</commit_message>
<xml_diff>
--- a/resultats_crete_a_crete.xlsx
+++ b/resultats_crete_a_crete.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -493,31 +493,181 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-c.XLSX</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.08668237445650107</v>
+        <v>0.06060952428349964</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-a.XLSX</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.08219353249770123</v>
+        <v>0.08931353045809942</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1131877105853007</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0.09804207332909698</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0.08668237445650107</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>0.08219353249770123</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-c.XLSX</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B13" t="n">
         <v>0.07733982644349879</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0.02745047319930016</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0.03119367244289961</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0.0259993461099004</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0.0593141764436993</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0.04366828172600101</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.04917877668509973</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.09146462191690219</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.07858205170039767</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-a.XLSX</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.07179453222410004</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-b.XLSX</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.0619274911100014</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-c.XLSX</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0.07747161397350055</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update file paths and enhance PRN to XLSX conversion in convert.py and matrice.py
</commit_message>
<xml_diff>
--- a/resultats_crete_a_crete.xlsx
+++ b/resultats_crete_a_crete.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,37 +443,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-a.xlsx</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.0229099980453995</v>
+        <v>0.02790779622080031</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-b.xlsx</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02831041432609993</v>
+        <v>0.02240072910350044</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.05µl-c.xlsx</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.03152538050700038</v>
+        <v>0.02534587985060099</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-a.xlsx</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -483,37 +483,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-b.xlsx</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06250011095490038</v>
+        <v>0.05770431497340134</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.08µl-c.xlsx</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.06060952428349964</v>
+        <v>0.05724856961239766</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-a.xlsx</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.08931353045809942</v>
+        <v>0.08092528591729931</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-b.xlsx</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -523,17 +523,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.12µl-c.xlsx</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.09804207332909698</v>
+        <v>0.09571180992369932</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-a.xlsx</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -543,7 +543,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-b.xlsx</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -553,37 +553,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 1 joints-0.1µl-c.xlsx</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.07733982644349879</v>
+        <v>0.08446305307899848</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-a.xlsx</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.02745047319930016</v>
+        <v>0.02330668131889979</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-b.xlsx</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.03119367244289961</v>
+        <v>0.02471835833000036</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.05µl-c.xlsx</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -593,7 +593,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-a.xlsx</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -603,27 +603,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-b.xlsx</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.04366828172600101</v>
+        <v>0.0386831090778994</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.08µl-c.xlsx</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.04917877668509973</v>
+        <v>0.04586121237549889</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-a.xlsx</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -633,41 +633,771 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-b.xlsx</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.07858205170039767</v>
+        <v>0.08031231295580099</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-a.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.12µl-c.xlsx</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0.07179453222410004</v>
+        <v>0.07028857573849834</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-b.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-a.xlsx</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>0.0619274911100014</v>
+        <v>0.07022726970080129</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-c.XLSX</t>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-b.xlsx</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0.07747161397350055</v>
+        <v>0.0615110828434986</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 Piston 2 joints-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0.07457701922120208</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.05µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>0.006208634560099568</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.05µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0.00230480917540099</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.05µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>0.005946887018099645</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.08µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>0.004851459189701757</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.08µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0.00945604683109913</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.08µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>0.005791327387100864</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.12µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.01012861411669874</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.12µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>0.009332133405202114</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.12µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0.01711439139170068</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.1µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>0.006237608799402494</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.1µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0.002555805007801837</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE neuf-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>0.005940843729099754</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.05µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>0.007485184747199725</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.05µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>0.00589855567439912</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.05µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>0.007777243707000281</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.08µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>0.01754445776739999</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.08µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>0.01691947589590015</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.08µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>0.01666811182249717</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.12µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>0.01740964108040188</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.12µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>0.01609029107499893</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.12µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0.01294869526260101</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.1µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0.02330351312440015</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.1µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0.0132804864365994</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole1 SGE Usagé-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0.0113570180548983</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.05µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0.05057010223030112</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.05µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>0.05366188503359837</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.05µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>0.0318464545942998</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.08µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>0.05011389895379992</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.08µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0.0600101473508996</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.08µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>0.06261151421050037</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.12µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>0.07306092010290044</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.12µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>0.09853656595729987</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.12µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>0.1012242470806015</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.1µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>0.0805514653710997</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.1µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>0.07602302033810027</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 1 joints-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>0.05534906920960125</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.05µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>0.02377068309080066</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.05µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>0.03131644183419979</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.05µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>0.03995059661929901</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.08µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>0.06005959236889957</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.08µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>0.04776025909530013</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.08µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>0.04642881261389853</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.12µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>0.1137349056474992</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.12µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>0.07733235819429929</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.12µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>0.1002179665818002</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.1µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>0.05555620427239916</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.1µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>0.09223355151809898</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 Piston 2 joints-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>0.087452723289001</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.05µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>0.02227767031059891</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.05µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>0.01335898495900167</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.05µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>0.00861701452430097</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.08µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>0.009574445160598799</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.08µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>0.01973913684770068</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.08µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>0.00620163558389919</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.12µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>0.0377091084243002</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.12µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>0.03863733270859981</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.12µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>0.04764727002419988</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.1µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>0.003813962213499167</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.1µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>0.004408800908899835</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE neuf-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>0.005621667563699972</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.05µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>0.02364662928169992</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.05µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>0.01738442407769902</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.05µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>0.01063066526990042</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.08µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>0.02535997174419968</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.08µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>0.005399909212700393</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.08µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>0.01198289344240067</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.12µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>0.01214411051210007</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.12µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>0.01525702924990036</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.12µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>0.006814742397798668</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.1µl-a.xlsx</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>0.01131478865080027</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.1µl-b.xlsx</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>0.00773025694240026</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Tests_amplitude  protocole2 SGE Usagé-0.1µl-c.xlsx</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>0.004778400121900006</v>
       </c>
     </row>
   </sheetData>

</xml_diff>